<commit_message>
Deposit product main (6cafd10): WB-13–21 + REAL-01
Sync latest klints_backend main into DEV client repo via deposit branch.
Preserves RELEASES, tag deploy workflow, claim/security docs, and production.env.
Code-only; no tag cut — FRA deploy still requires a new semver tag.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/sahil/CLIENT_BLOCKERS_AND_GAPS_BRIEF.xlsx
+++ b/docs/sahil/CLIENT_BLOCKERS_AND_GAPS_BRIEF.xlsx
@@ -524,7 +524,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Run 526 · headline 76.778 · PT-04 FAIL (kept for Fix story)</t>
+          <t>Run 526 snapshot still illustrative · writebacks LE-01/05/09, SP-07, PT-04 now Live OK (WB-08..WB-13); re-score after Approve to clear</t>
         </is>
       </c>
     </row>
@@ -796,22 +796,22 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>PT-04 FAIL on Fix; Handoff open in demo (QA can stay FAIL)</t>
+          <t>PT-04 was FAIL on Fix; Handoff demo may still open while QA FAIL</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Demo trap + Product gap</t>
+          <t>Closed for writeback (WB-11+WB-12) · Demo trap residual</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>PT-04 is money truth (Manago lifetime vs Shopify net / refunds). Product says writeback-class (Approve→execute). Code has no PT-04 writeback mapping — TRUE product gap. Demo: REQUIRE_HANDOFF_QA_PASS=False opens Handoff/stage while package QA is not PASS (Fix story). Production default True still requires QA PASS. Bypass ≠ writeback.</t>
+          <t>PT-04 money truth now has Fix Approve: stamps klints_net_ltv; re-run DCS PASSes when stamp ≈ Shopify net (WB-11+WB-12). Demo REQUIRE_HANDOFF_QA_PASS=False still opens Handoff while QA FAIL — bypass ≠ writeback.</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Client can walk Fix→Studio→QA→Handoff with PT-04 still FAIL. Cannot clear PT-04 via in-app writeback until mapping ships.</t>
+          <t>Client can clear PT-04 via Fix→Approve→re-score. Demo may still show Handoff open with FAIL for story.</t>
         </is>
       </c>
     </row>
@@ -823,22 +823,22 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>CheckMaster says Automated writeback; Approve disabled / missing</t>
+          <t>Some checks still say Automated writeback but Approve disabled</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>TRUE / Product gap</t>
+          <t>TRUE / Product gap (shrinking)</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Only CI-01, CC-03, WB-SHOP-01 are execute-ready. Many catalogue checks still claim writeback but have no mapping or are stubs.</t>
+          <t>Live OK now: CI-01, CC-03, WB-SHOP-01, LE-01 (WB-08), SP-07 (WB-09), LE-09 (WB-10), PT-04 (WB-11+12), LE-05 (WB-13). Still open/stub: CI-03, SP-01, LE-02, CI-05, PT-01/03, SP-03, CC-01/02, BR-01, LE-08; LE-04 intentional OFF.</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Client expects Fix→Approve→live Manago for those checks; path not wired yet.</t>
+          <t>Highest-pain gates LE-01/05/09/PT-04/SP-07 are executable; remaining catalogue promises still need mappings.</t>
         </is>
       </c>
     </row>
@@ -887,12 +887,12 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>SP-03/LE-09 style Manago data fixes + PT-01 line-item resolve (code). PT-04 intentionally left FAIL for Fix story.</t>
+          <t>SP-03/LE-09 style Manago data fixes + PT-01 join fix (code). PT-04 can now clear via writeback (WB-11+12) instead of staying FAIL forever.</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Headline can be high while Fix still shows PT-04.</t>
+          <t>Headline can be high; Fix can clear PT-04 when company writebacks enabled.</t>
         </is>
       </c>
     </row>
@@ -1925,32 +1925,32 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Stub</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>TRUE / Product gap</t>
+          <t>Live OK</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Event backfill stub only</t>
+          <t>Fix → Approve → PURCHASE event_ingest (WB-08); sandbox max_rows default 10</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Yes on several UCs</t>
+          <t>If FAIL, yes until PASS / re-score</t>
         </is>
       </c>
     </row>
@@ -2051,32 +2051,32 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>TRUE / Product gap + Demo trap</t>
+          <t>Live OK</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Money truth / refunds — should stop on writeback approval; no mapping → Fix cannot clear. Demo: Handoff unlocked via REQUIRE_HANDOFF_QA_PASS=False; production still wants QA PASS.</t>
+          <t>Stamps klints_net_ltv (WB-11); re-score PASSes when stamp ≈ Shopify net (WB-12). Prefer LE-09 PASS first.</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>YES for pilots/UC-06B when REQUIRE_PILOT_GATING_CHECKS=True; Handoff demo open when REQUIRE_HANDOFF_QA_PASS=False</t>
+          <t>Can clear via Approve→re-score; demo Handoff may still open while FAIL if REQUIRE_HANDOFF_QA_PASS=False</t>
         </is>
       </c>
     </row>
@@ -2093,32 +2093,32 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>TRUE / Product gap</t>
+          <t>Live OK</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>RETURN stream — fixed via ops script historically, not Fix Approve</t>
+          <t>RETURN event_ingest from shopify_only_return (WB-10); EVENT.INGEST batch ceiling</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Related to PT-04</t>
+          <t>Related to PT-04; clear via Approve→re-score</t>
         </is>
       </c>
     </row>
@@ -2177,32 +2177,32 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>TRUE / Product gap</t>
+          <t>Live OK</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Not execute-ready</t>
+          <t>Order-level PURCHASE gap event_ingest (WB-13); prefer Fix LE-05 over dual LE-01 Approve</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>UC-06B gate</t>
+          <t>UC-06B gate — clear via Approve→re-score</t>
         </is>
       </c>
     </row>
@@ -2387,32 +2387,32 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>TRUE / Product gap</t>
+          <t>Live OK</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>klints_ namespace collisions</t>
+          <t>Namespace collision rename (WB-09); re-run DCS after Approve</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>UC-23</t>
+          <t>UC-23 — clear via Approve→re-score</t>
         </is>
       </c>
     </row>
@@ -2747,22 +2747,22 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>No PT-04 mapping / not allowlisted</t>
+          <t>PT-04 was missing mapping; now Live OK (WB-11+12)</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>TRUE / Product gap</t>
+          <t>Closed (writeback shipped)</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Client expects Approve like other writeback checks</t>
+          <t>Fix → Approve stamps klints_net_ltv; re-run DCS to PASS</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Build PT-04 mapping OR manual Manago RETURN + re-score</t>
+          <t>Enable company writebacks; Approve → re-score. Demo may still keep FAIL for story.</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>REQUIRE_HANDOFF_QA_PASS=False (demo only) — stage/view Handoff while QA FAIL; QA/DCS tiles stay honest. Or clear PT-04 outside Klints WB / ship PT-04 writeback.</t>
+          <t>REQUIRE_HANDOFF_QA_PASS=False (demo only). Or clear PT-04 via Fix Approve (WB-11+12) then QA PASS.</t>
         </is>
       </c>
     </row>
@@ -3122,12 +3122,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>No mapping — GAP</t>
+          <t>Yes (Live OK — WB-11+12)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Kept for Fix story; clear via RETURN stream in Manago then re-score</t>
+          <t>Can clear via Fix Approve (klints_net_ltv stamp) then re-score; demo may keep FAIL for Fix story</t>
         </is>
       </c>
     </row>
@@ -3214,22 +3214,22 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Mark PT-04 writeback gap (G10). Demo policy shipped: REQUIRE_HANDOFF_QA_PASS=False opens Handoff while QA/PT-04 FAIL. Still need PT-04 mapping for real Fix clear, or keep FAIL as Fix-story evidence.</t>
+          <t>PT-04 writeback shipped (WB-11+12). Demo policy still: REQUIRE_HANDOFF_QA_PASS=False opens Handoff while QA/PT-04 FAIL. Prefer Approve→re-score to clear for real pilots.</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Build or Demo policy</t>
+          <t>Done (WB) · Demo policy residual</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Product + Eng</t>
+          <t>Product + Eng (done) / Demo eng</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Removes Fix→Handoff trap</t>
+          <t>Real Fix clear available; demo trap documented separately</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Ship writeback mappings for highest-pain gates: PT-04, LE-09, LE-01, LE-05, CC-01/02</t>
+          <t>Next writeback mappings for remaining pain: LE-02, CI-03, CC-01/02, CI-05 (LE-01/05/09, SP-07, PT-04 already Live)</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Fix→Approve matches CheckMaster promise</t>
+          <t>Fix→Approve matches remaining CheckMaster promises</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Enable stubs CI-03 / LE-01 only when transforms + capability status CONFIRMED</t>
+          <t>Enable stubs CI-03 / SP-01 only when transforms + capability status CONFIRMED (LE-01 already Live WB-08)</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">

</xml_diff>